<commit_message>
Commit- Orden, RFC CLIENTE, changes in doc base_cliente, detalles_individuales folder
</commit_message>
<xml_diff>
--- a/data/input/base_contratos.xlsx
+++ b/data/input/base_contratos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Soriana\00 - AUDITORIA 2020 - 2024\00 - Auditores\Oscar\Proyectos Python\Automation-Subarrenda\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BBE08E8-4E56-4063-AA4C-67AE4E8879F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473E6EB5-2D16-47F6-B8AA-D00507BA2A34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15840" xr2:uid="{0E8B9EC1-6715-4F8D-BBDE-46BF36F37EC3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9504" uniqueCount="2974">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9505" uniqueCount="2975">
   <si>
     <t>orden</t>
   </si>
@@ -8964,6 +8964,9 @@
   </si>
   <si>
     <t>208.50 METROS CUADRADOS</t>
+  </si>
+  <si>
+    <t>15/1/2015</t>
   </si>
 </sst>
 </file>
@@ -9345,6 +9348,7 @@
   <cols>
     <col min="6" max="7" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
@@ -14331,7 +14335,7 @@
     </row>
     <row r="50" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B50" t="s">
         <v>458</v>
@@ -14430,7 +14434,7 @@
     </row>
     <row r="51" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B51" t="s">
         <v>468</v>
@@ -14529,7 +14533,7 @@
     </row>
     <row r="52" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B52" t="s">
         <v>478</v>
@@ -14628,7 +14632,7 @@
     </row>
     <row r="53" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B53" t="s">
         <v>487</v>
@@ -14727,7 +14731,7 @@
     </row>
     <row r="54" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B54" t="s">
         <v>495</v>
@@ -14826,7 +14830,7 @@
     </row>
     <row r="55" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B55" t="s">
         <v>501</v>
@@ -14925,7 +14929,7 @@
     </row>
     <row r="56" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B56" t="s">
         <v>511</v>
@@ -15024,7 +15028,7 @@
     </row>
     <row r="57" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B57" t="s">
         <v>519</v>
@@ -15123,7 +15127,7 @@
     </row>
     <row r="58" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B58" t="s">
         <v>528</v>
@@ -15222,7 +15226,7 @@
     </row>
     <row r="59" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B59" t="s">
         <v>536</v>
@@ -15321,7 +15325,7 @@
     </row>
     <row r="60" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="B60" t="s">
         <v>544</v>
@@ -15420,7 +15424,7 @@
     </row>
     <row r="61" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="B61" t="s">
         <v>551</v>
@@ -15519,7 +15523,7 @@
     </row>
     <row r="62" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="B62" t="s">
         <v>558</v>
@@ -15618,7 +15622,7 @@
     </row>
     <row r="63" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A63">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="B63" t="s">
         <v>566</v>
@@ -15717,7 +15721,7 @@
     </row>
     <row r="64" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="B64" t="s">
         <v>575</v>
@@ -15816,7 +15820,7 @@
     </row>
     <row r="65" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="B65" t="s">
         <v>583</v>
@@ -15915,7 +15919,7 @@
     </row>
     <row r="66" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A66">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="B66" t="s">
         <v>591</v>
@@ -16014,7 +16018,7 @@
     </row>
     <row r="67" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="B67" t="s">
         <v>599</v>
@@ -16113,7 +16117,7 @@
     </row>
     <row r="68" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="B68" t="s">
         <v>606</v>
@@ -16212,7 +16216,7 @@
     </row>
     <row r="69" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="B69" t="s">
         <v>614</v>
@@ -16311,7 +16315,7 @@
     </row>
     <row r="70" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="B70" t="s">
         <v>626</v>
@@ -16410,7 +16414,7 @@
     </row>
     <row r="71" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="B71" t="s">
         <v>633</v>
@@ -16509,7 +16513,7 @@
     </row>
     <row r="72" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="B72" t="s">
         <v>639</v>
@@ -16608,7 +16612,7 @@
     </row>
     <row r="73" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="B73" t="s">
         <v>643</v>
@@ -16707,7 +16711,7 @@
     </row>
     <row r="74" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="B74" t="s">
         <v>652</v>
@@ -16806,7 +16810,7 @@
     </row>
     <row r="75" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="B75" t="s">
         <v>661</v>
@@ -16905,7 +16909,7 @@
     </row>
     <row r="76" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A76">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="B76" t="s">
         <v>670</v>
@@ -17004,7 +17008,7 @@
     </row>
     <row r="77" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="B77" t="s">
         <v>679</v>
@@ -17103,7 +17107,7 @@
     </row>
     <row r="78" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="B78" t="s">
         <v>686</v>
@@ -17202,7 +17206,7 @@
     </row>
     <row r="79" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="B79" t="s">
         <v>694</v>
@@ -17301,7 +17305,7 @@
     </row>
     <row r="80" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>401</v>
+        <v>394</v>
       </c>
       <c r="B80" t="s">
         <v>699</v>
@@ -17400,7 +17404,7 @@
     </row>
     <row r="81" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="B81" t="s">
         <v>703</v>
@@ -17499,7 +17503,7 @@
     </row>
     <row r="82" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="B82" t="s">
         <v>706</v>
@@ -17598,7 +17602,7 @@
     </row>
     <row r="83" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="B83" t="s">
         <v>710</v>
@@ -17697,7 +17701,7 @@
     </row>
     <row r="84" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="B84" t="s">
         <v>714</v>
@@ -17796,7 +17800,7 @@
     </row>
     <row r="85" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="B85" t="s">
         <v>718</v>
@@ -17895,7 +17899,7 @@
     </row>
     <row r="86" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="B86" t="s">
         <v>722</v>
@@ -17994,7 +17998,7 @@
     </row>
     <row r="87" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A87">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="B87" t="s">
         <v>727</v>
@@ -18093,7 +18097,7 @@
     </row>
     <row r="88" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A88">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="B88" t="s">
         <v>731</v>
@@ -18192,7 +18196,7 @@
     </row>
     <row r="89" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A89">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="B89" t="s">
         <v>735</v>
@@ -18291,7 +18295,7 @@
     </row>
     <row r="90" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A90">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="B90" t="s">
         <v>739</v>
@@ -18390,7 +18394,7 @@
     </row>
     <row r="91" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A91">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="B91" t="s">
         <v>743</v>
@@ -18489,7 +18493,7 @@
     </row>
     <row r="92" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A92">
-        <v>413</v>
+        <v>406</v>
       </c>
       <c r="B92" t="s">
         <v>747</v>
@@ -18588,7 +18592,7 @@
     </row>
     <row r="93" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A93">
-        <v>414</v>
+        <v>407</v>
       </c>
       <c r="B93" t="s">
         <v>751</v>
@@ -18687,7 +18691,7 @@
     </row>
     <row r="94" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A94">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="B94" t="s">
         <v>755</v>
@@ -18786,7 +18790,7 @@
     </row>
     <row r="95" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A95">
-        <v>416</v>
+        <v>409</v>
       </c>
       <c r="B95" t="s">
         <v>758</v>
@@ -18885,7 +18889,7 @@
     </row>
     <row r="96" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A96">
-        <v>417</v>
+        <v>410</v>
       </c>
       <c r="B96" t="s">
         <v>761</v>
@@ -18984,7 +18988,7 @@
     </row>
     <row r="97" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A97">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="B97" t="s">
         <v>765</v>
@@ -19083,7 +19087,7 @@
     </row>
     <row r="98" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>419</v>
+        <v>412</v>
       </c>
       <c r="B98" t="s">
         <v>768</v>
@@ -19182,7 +19186,7 @@
     </row>
     <row r="99" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A99">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="B99" t="s">
         <v>772</v>
@@ -19281,7 +19285,7 @@
     </row>
     <row r="100" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A100">
-        <v>421</v>
+        <v>414</v>
       </c>
       <c r="B100" t="s">
         <v>775</v>
@@ -19380,7 +19384,7 @@
     </row>
     <row r="101" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A101">
-        <v>422</v>
+        <v>415</v>
       </c>
       <c r="B101" t="s">
         <v>779</v>
@@ -19479,7 +19483,7 @@
     </row>
     <row r="102" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A102">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="B102" t="s">
         <v>783</v>
@@ -19578,7 +19582,7 @@
     </row>
     <row r="103" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A103">
-        <v>424</v>
+        <v>417</v>
       </c>
       <c r="B103" t="s">
         <v>786</v>
@@ -19677,7 +19681,7 @@
     </row>
     <row r="104" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A104">
-        <v>425</v>
+        <v>418</v>
       </c>
       <c r="B104" t="s">
         <v>790</v>
@@ -19776,7 +19780,7 @@
     </row>
     <row r="105" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A105">
-        <v>426</v>
+        <v>419</v>
       </c>
       <c r="B105" t="s">
         <v>793</v>
@@ -19875,7 +19879,7 @@
     </row>
     <row r="106" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A106">
-        <v>427</v>
+        <v>420</v>
       </c>
       <c r="B106" t="s">
         <v>797</v>
@@ -19974,7 +19978,7 @@
     </row>
     <row r="107" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A107">
-        <v>428</v>
+        <v>421</v>
       </c>
       <c r="B107" t="s">
         <v>800</v>
@@ -20073,7 +20077,7 @@
     </row>
     <row r="108" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A108">
-        <v>429</v>
+        <v>422</v>
       </c>
       <c r="B108" t="s">
         <v>803</v>
@@ -20172,7 +20176,7 @@
     </row>
     <row r="109" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A109">
-        <v>430</v>
+        <v>423</v>
       </c>
       <c r="B109" t="s">
         <v>807</v>
@@ -20271,7 +20275,7 @@
     </row>
     <row r="110" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A110">
-        <v>431</v>
+        <v>424</v>
       </c>
       <c r="B110" t="s">
         <v>811</v>
@@ -20370,7 +20374,7 @@
     </row>
     <row r="111" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A111">
-        <v>432</v>
+        <v>425</v>
       </c>
       <c r="B111" t="s">
         <v>814</v>
@@ -20469,7 +20473,7 @@
     </row>
     <row r="112" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A112">
-        <v>433</v>
+        <v>426</v>
       </c>
       <c r="B112" t="s">
         <v>818</v>
@@ -20568,7 +20572,7 @@
     </row>
     <row r="113" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A113">
-        <v>434</v>
+        <v>427</v>
       </c>
       <c r="B113" t="s">
         <v>821</v>
@@ -20667,7 +20671,7 @@
     </row>
     <row r="114" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A114">
-        <v>435</v>
+        <v>428</v>
       </c>
       <c r="B114" t="s">
         <v>825</v>
@@ -20766,7 +20770,7 @@
     </row>
     <row r="115" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A115">
-        <v>436</v>
+        <v>429</v>
       </c>
       <c r="B115" t="s">
         <v>828</v>
@@ -20865,7 +20869,7 @@
     </row>
     <row r="116" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A116">
-        <v>437</v>
+        <v>430</v>
       </c>
       <c r="B116" t="s">
         <v>832</v>
@@ -20964,7 +20968,7 @@
     </row>
     <row r="117" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A117">
-        <v>438</v>
+        <v>431</v>
       </c>
       <c r="B117" t="s">
         <v>836</v>
@@ -21063,7 +21067,7 @@
     </row>
     <row r="118" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A118">
-        <v>439</v>
+        <v>432</v>
       </c>
       <c r="B118" t="s">
         <v>840</v>
@@ -21162,7 +21166,7 @@
     </row>
     <row r="119" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A119">
-        <v>440</v>
+        <v>433</v>
       </c>
       <c r="B119" t="s">
         <v>844</v>
@@ -21261,7 +21265,7 @@
     </row>
     <row r="120" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A120">
-        <v>441</v>
+        <v>434</v>
       </c>
       <c r="B120" t="s">
         <v>847</v>
@@ -21360,7 +21364,7 @@
     </row>
     <row r="121" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A121">
-        <v>442</v>
+        <v>435</v>
       </c>
       <c r="B121" t="s">
         <v>850</v>
@@ -21459,7 +21463,7 @@
     </row>
     <row r="122" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A122">
-        <v>443</v>
+        <v>436</v>
       </c>
       <c r="B122" t="s">
         <v>854</v>
@@ -21558,7 +21562,7 @@
     </row>
     <row r="123" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A123">
-        <v>444</v>
+        <v>437</v>
       </c>
       <c r="B123" t="s">
         <v>857</v>
@@ -21657,7 +21661,7 @@
     </row>
     <row r="124" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A124">
-        <v>445</v>
+        <v>438</v>
       </c>
       <c r="B124" t="s">
         <v>860</v>
@@ -21756,7 +21760,7 @@
     </row>
     <row r="125" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A125">
-        <v>446</v>
+        <v>439</v>
       </c>
       <c r="B125" t="s">
         <v>863</v>
@@ -21855,7 +21859,7 @@
     </row>
     <row r="126" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A126">
-        <v>447</v>
+        <v>440</v>
       </c>
       <c r="B126" t="s">
         <v>866</v>
@@ -21954,7 +21958,7 @@
     </row>
     <row r="127" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A127">
-        <v>448</v>
+        <v>441</v>
       </c>
       <c r="B127" t="s">
         <v>870</v>
@@ -22053,7 +22057,7 @@
     </row>
     <row r="128" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A128">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="B128" t="s">
         <v>874</v>
@@ -22152,7 +22156,7 @@
     </row>
     <row r="129" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A129">
-        <v>450</v>
+        <v>443</v>
       </c>
       <c r="B129" t="s">
         <v>877</v>
@@ -22251,7 +22255,7 @@
     </row>
     <row r="130" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A130">
-        <v>451</v>
+        <v>444</v>
       </c>
       <c r="B130" t="s">
         <v>887</v>
@@ -22350,7 +22354,7 @@
     </row>
     <row r="131" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A131">
-        <v>452</v>
+        <v>445</v>
       </c>
       <c r="B131" t="s">
         <v>895</v>
@@ -22449,7 +22453,7 @@
     </row>
     <row r="132" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A132">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="B132" t="s">
         <v>902</v>
@@ -22548,7 +22552,7 @@
     </row>
     <row r="133" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A133">
-        <v>456</v>
+        <v>447</v>
       </c>
       <c r="B133" t="s">
         <v>909</v>
@@ -22647,7 +22651,7 @@
     </row>
     <row r="134" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A134">
-        <v>457</v>
+        <v>448</v>
       </c>
       <c r="B134" t="s">
         <v>916</v>
@@ -22746,7 +22750,7 @@
     </row>
     <row r="135" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A135">
-        <v>458</v>
+        <v>449</v>
       </c>
       <c r="B135" t="s">
         <v>924</v>
@@ -22845,7 +22849,7 @@
     </row>
     <row r="136" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A136">
-        <v>459</v>
+        <v>450</v>
       </c>
       <c r="B136" t="s">
         <v>932</v>
@@ -22944,7 +22948,7 @@
     </row>
     <row r="137" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A137">
-        <v>460</v>
+        <v>451</v>
       </c>
       <c r="B137" t="s">
         <v>939</v>
@@ -23043,7 +23047,7 @@
     </row>
     <row r="138" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A138">
-        <v>462</v>
+        <v>452</v>
       </c>
       <c r="B138" t="s">
         <v>942</v>
@@ -23142,7 +23146,7 @@
     </row>
     <row r="139" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A139">
-        <v>463</v>
+        <v>453</v>
       </c>
       <c r="B139" t="s">
         <v>949</v>
@@ -23340,7 +23344,7 @@
     </row>
     <row r="141" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A141">
-        <v>465</v>
+        <v>454</v>
       </c>
       <c r="B141" t="s">
         <v>960</v>
@@ -23439,7 +23443,7 @@
     </row>
     <row r="142" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A142">
-        <v>466</v>
+        <v>455</v>
       </c>
       <c r="B142" t="s">
         <v>969</v>
@@ -23538,7 +23542,7 @@
     </row>
     <row r="143" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A143">
-        <v>467</v>
+        <v>456</v>
       </c>
       <c r="B143" t="s">
         <v>977</v>
@@ -23637,7 +23641,7 @@
     </row>
     <row r="144" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A144">
-        <v>468</v>
+        <v>457</v>
       </c>
       <c r="B144" t="s">
         <v>984</v>
@@ -23736,7 +23740,7 @@
     </row>
     <row r="145" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A145">
-        <v>469</v>
+        <v>458</v>
       </c>
       <c r="B145" t="s">
         <v>991</v>
@@ -23835,7 +23839,7 @@
     </row>
     <row r="146" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A146">
-        <v>470</v>
+        <v>459</v>
       </c>
       <c r="B146" t="s">
         <v>995</v>
@@ -23934,7 +23938,7 @@
     </row>
     <row r="147" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A147">
-        <v>471</v>
+        <v>460</v>
       </c>
       <c r="B147" t="s">
         <v>1001</v>
@@ -24033,7 +24037,7 @@
     </row>
     <row r="148" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A148">
-        <v>472</v>
+        <v>461</v>
       </c>
       <c r="B148" t="s">
         <v>1009</v>
@@ -24132,7 +24136,7 @@
     </row>
     <row r="149" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A149">
-        <v>473</v>
+        <v>462</v>
       </c>
       <c r="B149" t="s">
         <v>1016</v>
@@ -24231,7 +24235,7 @@
     </row>
     <row r="150" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A150">
-        <v>474</v>
+        <v>463</v>
       </c>
       <c r="B150" t="s">
         <v>1022</v>
@@ -24330,7 +24334,7 @@
     </row>
     <row r="151" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A151">
-        <v>475</v>
+        <v>464</v>
       </c>
       <c r="B151" t="s">
         <v>1031</v>
@@ -24429,7 +24433,7 @@
     </row>
     <row r="152" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A152">
-        <v>476</v>
+        <v>465</v>
       </c>
       <c r="B152" t="s">
         <v>1040</v>
@@ -24528,7 +24532,7 @@
     </row>
     <row r="153" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A153">
-        <v>477</v>
+        <v>466</v>
       </c>
       <c r="B153" t="s">
         <v>1050</v>
@@ -24627,7 +24631,7 @@
     </row>
     <row r="154" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A154">
-        <v>478</v>
+        <v>467</v>
       </c>
       <c r="B154" t="s">
         <v>1058</v>
@@ -24726,7 +24730,7 @@
     </row>
     <row r="155" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A155">
-        <v>479</v>
+        <v>468</v>
       </c>
       <c r="B155" t="s">
         <v>1067</v>
@@ -24825,7 +24829,7 @@
     </row>
     <row r="156" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A156">
-        <v>480</v>
+        <v>469</v>
       </c>
       <c r="B156" t="s">
         <v>1076</v>
@@ -24924,7 +24928,7 @@
     </row>
     <row r="157" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A157">
-        <v>481</v>
+        <v>470</v>
       </c>
       <c r="B157" t="s">
         <v>1084</v>
@@ -25023,7 +25027,7 @@
     </row>
     <row r="158" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A158">
-        <v>482</v>
+        <v>471</v>
       </c>
       <c r="B158" t="s">
         <v>1092</v>
@@ -25122,7 +25126,7 @@
     </row>
     <row r="159" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A159">
-        <v>483</v>
+        <v>472</v>
       </c>
       <c r="B159" t="s">
         <v>1101</v>
@@ -25221,7 +25225,7 @@
     </row>
     <row r="160" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A160">
-        <v>484</v>
+        <v>473</v>
       </c>
       <c r="B160" t="s">
         <v>1110</v>
@@ -25320,7 +25324,7 @@
     </row>
     <row r="161" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A161">
-        <v>485</v>
+        <v>474</v>
       </c>
       <c r="B161" t="s">
         <v>1117</v>
@@ -25419,7 +25423,7 @@
     </row>
     <row r="162" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A162">
-        <v>486</v>
+        <v>475</v>
       </c>
       <c r="B162" t="s">
         <v>1125</v>
@@ -25518,7 +25522,7 @@
     </row>
     <row r="163" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A163">
-        <v>488</v>
+        <v>476</v>
       </c>
       <c r="B163" t="s">
         <v>1132</v>
@@ -25617,7 +25621,7 @@
     </row>
     <row r="164" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A164">
-        <v>489</v>
+        <v>477</v>
       </c>
       <c r="B164" t="s">
         <v>1140</v>
@@ -25716,7 +25720,7 @@
     </row>
     <row r="165" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A165">
-        <v>490</v>
+        <v>478</v>
       </c>
       <c r="B165" t="s">
         <v>1144</v>
@@ -25815,7 +25819,7 @@
     </row>
     <row r="166" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A166">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="B166" t="s">
         <v>1151</v>
@@ -25914,7 +25918,7 @@
     </row>
     <row r="167" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A167">
-        <v>494</v>
+        <v>480</v>
       </c>
       <c r="B167" t="s">
         <v>1155</v>
@@ -26013,7 +26017,7 @@
     </row>
     <row r="168" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A168">
-        <v>495</v>
+        <v>481</v>
       </c>
       <c r="B168" t="s">
         <v>1159</v>
@@ -26112,7 +26116,7 @@
     </row>
     <row r="169" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A169">
-        <v>496</v>
+        <v>482</v>
       </c>
       <c r="B169" t="s">
         <v>1162</v>
@@ -26211,7 +26215,7 @@
     </row>
     <row r="170" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A170">
-        <v>497</v>
+        <v>483</v>
       </c>
       <c r="B170" t="s">
         <v>1167</v>
@@ -26310,7 +26314,7 @@
     </row>
     <row r="171" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A171">
-        <v>498</v>
+        <v>484</v>
       </c>
       <c r="B171" t="s">
         <v>1173</v>
@@ -26409,7 +26413,7 @@
     </row>
     <row r="172" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A172">
-        <v>499</v>
+        <v>485</v>
       </c>
       <c r="B172" t="s">
         <v>1178</v>
@@ -26508,7 +26512,7 @@
     </row>
     <row r="173" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A173">
-        <v>500</v>
+        <v>486</v>
       </c>
       <c r="B173" t="s">
         <v>1184</v>
@@ -26607,7 +26611,7 @@
     </row>
     <row r="174" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A174">
-        <v>501</v>
+        <v>487</v>
       </c>
       <c r="B174" t="s">
         <v>1190</v>
@@ -26706,7 +26710,7 @@
     </row>
     <row r="175" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A175">
-        <v>502</v>
+        <v>488</v>
       </c>
       <c r="B175" t="s">
         <v>1195</v>
@@ -26805,7 +26809,7 @@
     </row>
     <row r="176" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A176">
-        <v>503</v>
+        <v>489</v>
       </c>
       <c r="B176" t="s">
         <v>1201</v>
@@ -26904,7 +26908,7 @@
     </row>
     <row r="177" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A177">
-        <v>505</v>
+        <v>490</v>
       </c>
       <c r="B177" t="s">
         <v>1211</v>
@@ -27003,7 +27007,7 @@
     </row>
     <row r="178" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A178">
-        <v>506</v>
+        <v>491</v>
       </c>
       <c r="B178" t="s">
         <v>1222</v>
@@ -27102,7 +27106,7 @@
     </row>
     <row r="179" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A179">
-        <v>507</v>
+        <v>492</v>
       </c>
       <c r="B179" t="s">
         <v>1230</v>
@@ -27201,7 +27205,7 @@
     </row>
     <row r="180" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A180">
-        <v>508</v>
+        <v>493</v>
       </c>
       <c r="B180" t="s">
         <v>1237</v>
@@ -27300,7 +27304,7 @@
     </row>
     <row r="181" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A181">
-        <v>509</v>
+        <v>494</v>
       </c>
       <c r="B181" t="s">
         <v>1248</v>
@@ -27399,7 +27403,7 @@
     </row>
     <row r="182" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A182">
-        <v>510</v>
+        <v>495</v>
       </c>
       <c r="B182" t="s">
         <v>1252</v>
@@ -27498,7 +27502,7 @@
     </row>
     <row r="183" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A183">
-        <v>511</v>
+        <v>496</v>
       </c>
       <c r="B183" t="s">
         <v>1262</v>
@@ -27597,7 +27601,7 @@
     </row>
     <row r="184" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A184">
-        <v>512</v>
+        <v>497</v>
       </c>
       <c r="B184" t="s">
         <v>1273</v>
@@ -27696,7 +27700,7 @@
     </row>
     <row r="185" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A185">
-        <v>513</v>
+        <v>498</v>
       </c>
       <c r="B185" t="s">
         <v>1282</v>
@@ -27795,7 +27799,7 @@
     </row>
     <row r="186" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A186">
-        <v>514</v>
+        <v>499</v>
       </c>
       <c r="B186" t="s">
         <v>1292</v>
@@ -27894,7 +27898,7 @@
     </row>
     <row r="187" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A187">
-        <v>515</v>
+        <v>500</v>
       </c>
       <c r="B187" t="s">
         <v>1298</v>
@@ -27993,7 +27997,7 @@
     </row>
     <row r="188" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A188">
-        <v>516</v>
+        <v>501</v>
       </c>
       <c r="B188" t="s">
         <v>1306</v>
@@ -28092,7 +28096,7 @@
     </row>
     <row r="189" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A189">
-        <v>517</v>
+        <v>502</v>
       </c>
       <c r="B189" t="s">
         <v>1316</v>
@@ -28191,7 +28195,7 @@
     </row>
     <row r="190" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A190">
-        <v>518</v>
+        <v>503</v>
       </c>
       <c r="B190" t="s">
         <v>1321</v>
@@ -28290,7 +28294,7 @@
     </row>
     <row r="191" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A191">
-        <v>519</v>
+        <v>504</v>
       </c>
       <c r="B191" t="s">
         <v>1332</v>
@@ -28389,7 +28393,7 @@
     </row>
     <row r="192" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A192">
-        <v>520</v>
+        <v>505</v>
       </c>
       <c r="B192" t="s">
         <v>1341</v>
@@ -28488,7 +28492,7 @@
     </row>
     <row r="193" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A193">
-        <v>521</v>
+        <v>506</v>
       </c>
       <c r="B193" t="s">
         <v>1352</v>
@@ -28587,7 +28591,7 @@
     </row>
     <row r="194" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A194">
-        <v>522</v>
+        <v>507</v>
       </c>
       <c r="B194" t="s">
         <v>1362</v>
@@ -28686,7 +28690,7 @@
     </row>
     <row r="195" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A195">
-        <v>523</v>
+        <v>508</v>
       </c>
       <c r="B195" t="s">
         <v>1367</v>
@@ -28785,7 +28789,7 @@
     </row>
     <row r="196" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A196">
-        <v>524</v>
+        <v>509</v>
       </c>
       <c r="B196" t="s">
         <v>1378</v>
@@ -28884,7 +28888,7 @@
     </row>
     <row r="197" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A197">
-        <v>525</v>
+        <v>510</v>
       </c>
       <c r="B197" t="s">
         <v>1384</v>
@@ -28983,7 +28987,7 @@
     </row>
     <row r="198" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A198">
-        <v>526</v>
+        <v>511</v>
       </c>
       <c r="B198" t="s">
         <v>1388</v>
@@ -29082,7 +29086,7 @@
     </row>
     <row r="199" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A199">
-        <v>527</v>
+        <v>512</v>
       </c>
       <c r="B199" t="s">
         <v>1397</v>
@@ -29181,7 +29185,7 @@
     </row>
     <row r="200" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A200">
-        <v>528</v>
+        <v>513</v>
       </c>
       <c r="B200" t="s">
         <v>1407</v>
@@ -29280,7 +29284,7 @@
     </row>
     <row r="201" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A201">
-        <v>529</v>
+        <v>514</v>
       </c>
       <c r="B201" t="s">
         <v>1417</v>
@@ -29379,7 +29383,7 @@
     </row>
     <row r="202" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A202">
-        <v>531</v>
+        <v>515</v>
       </c>
       <c r="B202" t="s">
         <v>1426</v>
@@ -29478,7 +29482,7 @@
     </row>
     <row r="203" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A203">
-        <v>532</v>
+        <v>516</v>
       </c>
       <c r="B203" t="s">
         <v>1433</v>
@@ -29577,7 +29581,7 @@
     </row>
     <row r="204" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A204">
-        <v>533</v>
+        <v>517</v>
       </c>
       <c r="B204" t="s">
         <v>1436</v>
@@ -29676,7 +29680,7 @@
     </row>
     <row r="205" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A205">
-        <v>534</v>
+        <v>518</v>
       </c>
       <c r="B205" t="s">
         <v>1439</v>
@@ -29775,7 +29779,7 @@
     </row>
     <row r="206" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A206">
-        <v>536</v>
+        <v>519</v>
       </c>
       <c r="B206" t="s">
         <v>1446</v>
@@ -29874,7 +29878,7 @@
     </row>
     <row r="207" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A207">
-        <v>537</v>
+        <v>520</v>
       </c>
       <c r="B207" t="s">
         <v>1451</v>
@@ -29973,7 +29977,7 @@
     </row>
     <row r="208" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A208">
-        <v>538</v>
+        <v>521</v>
       </c>
       <c r="B208" t="s">
         <v>1455</v>
@@ -30072,7 +30076,7 @@
     </row>
     <row r="209" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A209">
-        <v>539</v>
+        <v>522</v>
       </c>
       <c r="B209" t="s">
         <v>1464</v>
@@ -30171,7 +30175,7 @@
     </row>
     <row r="210" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A210">
-        <v>540</v>
+        <v>523</v>
       </c>
       <c r="B210" t="s">
         <v>1472</v>
@@ -30270,7 +30274,7 @@
     </row>
     <row r="211" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A211">
-        <v>541</v>
+        <v>524</v>
       </c>
       <c r="B211" t="s">
         <v>1480</v>
@@ -30369,7 +30373,7 @@
     </row>
     <row r="212" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A212">
-        <v>542</v>
+        <v>525</v>
       </c>
       <c r="B212" t="s">
         <v>1488</v>
@@ -30468,7 +30472,7 @@
     </row>
     <row r="213" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A213">
-        <v>543</v>
+        <v>526</v>
       </c>
       <c r="B213" t="s">
         <v>1497</v>
@@ -30567,7 +30571,7 @@
     </row>
     <row r="214" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A214">
-        <v>544</v>
+        <v>527</v>
       </c>
       <c r="B214" t="s">
         <v>1505</v>
@@ -30666,7 +30670,7 @@
     </row>
     <row r="215" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A215">
-        <v>545</v>
+        <v>528</v>
       </c>
       <c r="B215" t="s">
         <v>1507</v>
@@ -30765,7 +30769,7 @@
     </row>
     <row r="216" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A216">
-        <v>546</v>
+        <v>529</v>
       </c>
       <c r="B216" t="s">
         <v>1512</v>
@@ -30864,7 +30868,7 @@
     </row>
     <row r="217" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A217">
-        <v>547</v>
+        <v>530</v>
       </c>
       <c r="B217" t="s">
         <v>1523</v>
@@ -30963,7 +30967,7 @@
     </row>
     <row r="218" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A218">
-        <v>548</v>
+        <v>531</v>
       </c>
       <c r="B218" t="s">
         <v>1533</v>
@@ -31062,7 +31066,7 @@
     </row>
     <row r="219" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A219">
-        <v>549</v>
+        <v>532</v>
       </c>
       <c r="B219" t="s">
         <v>1541</v>
@@ -31161,7 +31165,7 @@
     </row>
     <row r="220" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A220">
-        <v>550</v>
+        <v>533</v>
       </c>
       <c r="B220" t="s">
         <v>1548</v>
@@ -31260,7 +31264,7 @@
     </row>
     <row r="221" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A221">
-        <v>551</v>
+        <v>534</v>
       </c>
       <c r="B221" t="s">
         <v>1556</v>
@@ -31359,7 +31363,7 @@
     </row>
     <row r="222" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A222">
-        <v>552</v>
+        <v>535</v>
       </c>
       <c r="B222" t="s">
         <v>1565</v>
@@ -31458,7 +31462,7 @@
     </row>
     <row r="223" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A223">
-        <v>553</v>
+        <v>536</v>
       </c>
       <c r="B223" t="s">
         <v>1574</v>
@@ -31557,7 +31561,7 @@
     </row>
     <row r="224" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A224">
-        <v>554</v>
+        <v>537</v>
       </c>
       <c r="B224" t="s">
         <v>1583</v>
@@ -31656,7 +31660,7 @@
     </row>
     <row r="225" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A225">
-        <v>555</v>
+        <v>538</v>
       </c>
       <c r="B225" t="s">
         <v>1594</v>
@@ -31755,7 +31759,7 @@
     </row>
     <row r="226" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A226">
-        <v>557</v>
+        <v>539</v>
       </c>
       <c r="B226" t="s">
         <v>1604</v>
@@ -31854,7 +31858,7 @@
     </row>
     <row r="227" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A227">
-        <v>558</v>
+        <v>540</v>
       </c>
       <c r="B227" t="s">
         <v>1615</v>
@@ -31953,7 +31957,7 @@
     </row>
     <row r="228" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A228">
-        <v>559</v>
+        <v>541</v>
       </c>
       <c r="B228" t="s">
         <v>1626</v>
@@ -32052,7 +32056,7 @@
     </row>
     <row r="229" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A229">
-        <v>560</v>
+        <v>542</v>
       </c>
       <c r="B229" t="s">
         <v>1635</v>
@@ -32151,7 +32155,7 @@
     </row>
     <row r="230" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A230">
-        <v>561</v>
+        <v>543</v>
       </c>
       <c r="B230" t="s">
         <v>1646</v>
@@ -32250,7 +32254,7 @@
     </row>
     <row r="231" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A231">
-        <v>562</v>
+        <v>544</v>
       </c>
       <c r="B231" t="s">
         <v>1657</v>
@@ -32349,7 +32353,7 @@
     </row>
     <row r="232" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A232">
-        <v>563</v>
+        <v>545</v>
       </c>
       <c r="B232" t="s">
         <v>1663</v>
@@ -32448,7 +32452,7 @@
     </row>
     <row r="233" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A233">
-        <v>564</v>
+        <v>546</v>
       </c>
       <c r="B233" t="s">
         <v>1671</v>
@@ -32547,7 +32551,7 @@
     </row>
     <row r="234" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A234">
-        <v>565</v>
+        <v>547</v>
       </c>
       <c r="B234" t="s">
         <v>1682</v>
@@ -32646,7 +32650,7 @@
     </row>
     <row r="235" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A235">
-        <v>566</v>
+        <v>548</v>
       </c>
       <c r="B235" t="s">
         <v>1693</v>
@@ -32745,7 +32749,7 @@
     </row>
     <row r="236" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A236">
-        <v>567</v>
+        <v>549</v>
       </c>
       <c r="B236" t="s">
         <v>1703</v>
@@ -32844,7 +32848,7 @@
     </row>
     <row r="237" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A237">
-        <v>569</v>
+        <v>550</v>
       </c>
       <c r="B237" t="s">
         <v>1712</v>
@@ -32943,7 +32947,7 @@
     </row>
     <row r="238" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A238">
-        <v>570</v>
+        <v>551</v>
       </c>
       <c r="B238" t="s">
         <v>1718</v>
@@ -33042,7 +33046,7 @@
     </row>
     <row r="239" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A239">
-        <v>571</v>
+        <v>552</v>
       </c>
       <c r="B239" t="s">
         <v>1723</v>
@@ -33141,7 +33145,7 @@
     </row>
     <row r="240" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A240">
-        <v>572</v>
+        <v>553</v>
       </c>
       <c r="B240" t="s">
         <v>1734</v>
@@ -33240,7 +33244,7 @@
     </row>
     <row r="241" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A241">
-        <v>573</v>
+        <v>554</v>
       </c>
       <c r="B241" t="s">
         <v>1744</v>
@@ -33339,7 +33343,7 @@
     </row>
     <row r="242" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A242">
-        <v>574</v>
+        <v>555</v>
       </c>
       <c r="B242" t="s">
         <v>1754</v>
@@ -33438,7 +33442,7 @@
     </row>
     <row r="243" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A243">
-        <v>578</v>
+        <v>556</v>
       </c>
       <c r="B243" t="s">
         <v>1763</v>
@@ -33537,7 +33541,7 @@
     </row>
     <row r="244" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A244">
-        <v>580</v>
+        <v>557</v>
       </c>
       <c r="B244" t="s">
         <v>1772</v>
@@ -33636,7 +33640,7 @@
     </row>
     <row r="245" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A245">
-        <v>581</v>
+        <v>558</v>
       </c>
       <c r="B245" t="s">
         <v>1781</v>
@@ -33735,7 +33739,7 @@
     </row>
     <row r="246" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A246">
-        <v>582</v>
+        <v>559</v>
       </c>
       <c r="B246" t="s">
         <v>1791</v>
@@ -33834,7 +33838,7 @@
     </row>
     <row r="247" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A247">
-        <v>583</v>
+        <v>560</v>
       </c>
       <c r="B247" t="s">
         <v>1802</v>
@@ -33933,7 +33937,7 @@
     </row>
     <row r="248" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A248">
-        <v>585</v>
+        <v>561</v>
       </c>
       <c r="B248" t="s">
         <v>1813</v>
@@ -33944,8 +33948,8 @@
       <c r="D248" t="s">
         <v>1814</v>
       </c>
-      <c r="F248" s="1">
-        <v>42019</v>
+      <c r="F248" s="1" t="s">
+        <v>2974</v>
       </c>
       <c r="G248" s="1">
         <v>47285</v>
@@ -34032,7 +34036,7 @@
     </row>
     <row r="249" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A249">
-        <v>586</v>
+        <v>562</v>
       </c>
       <c r="B249" t="s">
         <v>1820</v>
@@ -34131,7 +34135,7 @@
     </row>
     <row r="250" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A250">
-        <v>587</v>
+        <v>563</v>
       </c>
       <c r="B250" t="s">
         <v>1826</v>
@@ -34230,7 +34234,7 @@
     </row>
     <row r="251" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A251">
-        <v>588</v>
+        <v>564</v>
       </c>
       <c r="B251" t="s">
         <v>1837</v>
@@ -34329,7 +34333,7 @@
     </row>
     <row r="252" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A252">
-        <v>589</v>
+        <v>565</v>
       </c>
       <c r="B252" t="s">
         <v>1846</v>
@@ -34428,7 +34432,7 @@
     </row>
     <row r="253" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A253">
-        <v>590</v>
+        <v>566</v>
       </c>
       <c r="B253" t="s">
         <v>1855</v>
@@ -34527,7 +34531,7 @@
     </row>
     <row r="254" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A254">
-        <v>591</v>
+        <v>567</v>
       </c>
       <c r="B254" t="s">
         <v>1859</v>
@@ -34626,7 +34630,7 @@
     </row>
     <row r="255" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A255">
-        <v>592</v>
+        <v>568</v>
       </c>
       <c r="B255" t="s">
         <v>1868</v>
@@ -34725,7 +34729,7 @@
     </row>
     <row r="256" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A256">
-        <v>593</v>
+        <v>569</v>
       </c>
       <c r="B256" t="s">
         <v>1875</v>
@@ -34824,7 +34828,7 @@
     </row>
     <row r="257" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A257">
-        <v>594</v>
+        <v>570</v>
       </c>
       <c r="B257" t="s">
         <v>1886</v>
@@ -34923,7 +34927,7 @@
     </row>
     <row r="258" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A258">
-        <v>595</v>
+        <v>571</v>
       </c>
       <c r="B258" t="s">
         <v>1895</v>
@@ -35022,7 +35026,7 @@
     </row>
     <row r="259" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A259">
-        <v>596</v>
+        <v>572</v>
       </c>
       <c r="B259" t="s">
         <v>1903</v>
@@ -35121,7 +35125,7 @@
     </row>
     <row r="260" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A260">
-        <v>597</v>
+        <v>573</v>
       </c>
       <c r="B260" t="s">
         <v>1908</v>
@@ -35220,7 +35224,7 @@
     </row>
     <row r="261" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A261">
-        <v>598</v>
+        <v>574</v>
       </c>
       <c r="B261" t="s">
         <v>1917</v>
@@ -35319,7 +35323,7 @@
     </row>
     <row r="262" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A262">
-        <v>600</v>
+        <v>575</v>
       </c>
       <c r="B262" t="s">
         <v>1921</v>
@@ -35418,7 +35422,7 @@
     </row>
     <row r="263" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A263">
-        <v>601</v>
+        <v>576</v>
       </c>
       <c r="B263" t="s">
         <v>1927</v>
@@ -35517,7 +35521,7 @@
     </row>
     <row r="264" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A264">
-        <v>602</v>
+        <v>577</v>
       </c>
       <c r="B264" t="s">
         <v>1932</v>
@@ -35616,7 +35620,7 @@
     </row>
     <row r="265" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A265">
-        <v>603</v>
+        <v>578</v>
       </c>
       <c r="B265" t="s">
         <v>1940</v>
@@ -35715,7 +35719,7 @@
     </row>
     <row r="266" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A266">
-        <v>604</v>
+        <v>579</v>
       </c>
       <c r="B266" t="s">
         <v>1946</v>
@@ -35814,7 +35818,7 @@
     </row>
     <row r="267" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A267">
-        <v>606</v>
+        <v>580</v>
       </c>
       <c r="B267" t="s">
         <v>1954</v>
@@ -35913,7 +35917,7 @@
     </row>
     <row r="268" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A268">
-        <v>607</v>
+        <v>581</v>
       </c>
       <c r="B268" t="s">
         <v>1963</v>
@@ -36012,7 +36016,7 @@
     </row>
     <row r="269" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A269">
-        <v>609</v>
+        <v>582</v>
       </c>
       <c r="B269" t="s">
         <v>1973</v>
@@ -36111,7 +36115,7 @@
     </row>
     <row r="270" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A270">
-        <v>610</v>
+        <v>583</v>
       </c>
       <c r="B270" t="s">
         <v>1983</v>
@@ -36210,7 +36214,7 @@
     </row>
     <row r="271" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A271">
-        <v>611</v>
+        <v>584</v>
       </c>
       <c r="B271" t="s">
         <v>1991</v>
@@ -36309,7 +36313,7 @@
     </row>
     <row r="272" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A272">
-        <v>612</v>
+        <v>585</v>
       </c>
       <c r="B272" t="s">
         <v>1999</v>
@@ -36408,7 +36412,7 @@
     </row>
     <row r="273" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A273">
-        <v>613</v>
+        <v>586</v>
       </c>
       <c r="B273" t="s">
         <v>2007</v>
@@ -36507,7 +36511,7 @@
     </row>
     <row r="274" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A274">
-        <v>614</v>
+        <v>587</v>
       </c>
       <c r="B274" t="s">
         <v>2011</v>
@@ -36606,7 +36610,7 @@
     </row>
     <row r="275" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A275">
-        <v>615</v>
+        <v>588</v>
       </c>
       <c r="B275" t="s">
         <v>2016</v>
@@ -36705,7 +36709,7 @@
     </row>
     <row r="276" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A276">
-        <v>616</v>
+        <v>589</v>
       </c>
       <c r="B276" t="s">
         <v>2021</v>
@@ -36804,7 +36808,7 @@
     </row>
     <row r="277" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A277">
-        <v>618</v>
+        <v>590</v>
       </c>
       <c r="B277" t="s">
         <v>2026</v>
@@ -36903,7 +36907,7 @@
     </row>
     <row r="278" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A278">
-        <v>619</v>
+        <v>591</v>
       </c>
       <c r="B278" t="s">
         <v>2032</v>
@@ -37002,7 +37006,7 @@
     </row>
     <row r="279" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A279">
-        <v>620</v>
+        <v>592</v>
       </c>
       <c r="B279" t="s">
         <v>2036</v>
@@ -37101,7 +37105,7 @@
     </row>
     <row r="280" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A280">
-        <v>622</v>
+        <v>593</v>
       </c>
       <c r="B280" t="s">
         <v>2047</v>
@@ -37200,7 +37204,7 @@
     </row>
     <row r="281" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A281">
-        <v>623</v>
+        <v>594</v>
       </c>
       <c r="B281" t="s">
         <v>2056</v>
@@ -37299,7 +37303,7 @@
     </row>
     <row r="282" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A282">
-        <v>624</v>
+        <v>595</v>
       </c>
       <c r="B282" t="s">
         <v>2065</v>
@@ -37398,7 +37402,7 @@
     </row>
     <row r="283" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A283">
-        <v>625</v>
+        <v>596</v>
       </c>
       <c r="B283" t="s">
         <v>2070</v>
@@ -37497,7 +37501,7 @@
     </row>
     <row r="284" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A284">
-        <v>626</v>
+        <v>597</v>
       </c>
       <c r="B284" t="s">
         <v>2080</v>
@@ -37596,7 +37600,7 @@
     </row>
     <row r="285" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A285">
-        <v>627</v>
+        <v>598</v>
       </c>
       <c r="B285" t="s">
         <v>2088</v>
@@ -37695,7 +37699,7 @@
     </row>
     <row r="286" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A286">
-        <v>629</v>
+        <v>599</v>
       </c>
       <c r="B286" t="s">
         <v>2092</v>
@@ -37794,7 +37798,7 @@
     </row>
     <row r="287" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A287">
-        <v>630</v>
+        <v>600</v>
       </c>
       <c r="B287" t="s">
         <v>2103</v>
@@ -37893,7 +37897,7 @@
     </row>
     <row r="288" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A288">
-        <v>631</v>
+        <v>601</v>
       </c>
       <c r="B288" t="s">
         <v>2110</v>
@@ -37992,7 +37996,7 @@
     </row>
     <row r="289" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A289">
-        <v>632</v>
+        <v>602</v>
       </c>
       <c r="B289" t="s">
         <v>2122</v>
@@ -38091,7 +38095,7 @@
     </row>
     <row r="290" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A290">
-        <v>633</v>
+        <v>603</v>
       </c>
       <c r="B290" t="s">
         <v>2128</v>
@@ -38190,7 +38194,7 @@
     </row>
     <row r="291" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A291">
-        <v>634</v>
+        <v>604</v>
       </c>
       <c r="B291" t="s">
         <v>2132</v>
@@ -38289,7 +38293,7 @@
     </row>
     <row r="292" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A292">
-        <v>635</v>
+        <v>605</v>
       </c>
       <c r="B292" t="s">
         <v>2138</v>
@@ -38388,7 +38392,7 @@
     </row>
     <row r="293" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A293">
-        <v>638</v>
+        <v>606</v>
       </c>
       <c r="B293" t="s">
         <v>2147</v>
@@ -38487,7 +38491,7 @@
     </row>
     <row r="294" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A294">
-        <v>639</v>
+        <v>607</v>
       </c>
       <c r="B294" t="s">
         <v>2157</v>
@@ -38586,7 +38590,7 @@
     </row>
     <row r="295" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A295">
-        <v>640</v>
+        <v>608</v>
       </c>
       <c r="B295" t="s">
         <v>2164</v>
@@ -38685,7 +38689,7 @@
     </row>
     <row r="296" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A296">
-        <v>641</v>
+        <v>609</v>
       </c>
       <c r="B296" t="s">
         <v>2171</v>
@@ -38784,7 +38788,7 @@
     </row>
     <row r="297" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A297">
-        <v>642</v>
+        <v>610</v>
       </c>
       <c r="B297" t="s">
         <v>2181</v>
@@ -38883,7 +38887,7 @@
     </row>
     <row r="298" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A298">
-        <v>643</v>
+        <v>611</v>
       </c>
       <c r="B298" t="s">
         <v>2190</v>
@@ -38982,7 +38986,7 @@
     </row>
     <row r="299" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A299">
-        <v>644</v>
+        <v>612</v>
       </c>
       <c r="B299" t="s">
         <v>2200</v>
@@ -39081,7 +39085,7 @@
     </row>
     <row r="300" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A300">
-        <v>645</v>
+        <v>613</v>
       </c>
       <c r="B300" t="s">
         <v>2207</v>
@@ -39180,7 +39184,7 @@
     </row>
     <row r="301" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A301">
-        <v>646</v>
+        <v>614</v>
       </c>
       <c r="B301" t="s">
         <v>2212</v>
@@ -39279,7 +39283,7 @@
     </row>
     <row r="302" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A302">
-        <v>647</v>
+        <v>615</v>
       </c>
       <c r="B302" t="s">
         <v>2216</v>
@@ -39378,7 +39382,7 @@
     </row>
     <row r="303" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A303">
-        <v>648</v>
+        <v>616</v>
       </c>
       <c r="B303" t="s">
         <v>2220</v>
@@ -39477,7 +39481,7 @@
     </row>
     <row r="304" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A304">
-        <v>649</v>
+        <v>617</v>
       </c>
       <c r="B304" t="s">
         <v>2225</v>
@@ -39576,7 +39580,7 @@
     </row>
     <row r="305" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A305">
-        <v>650</v>
+        <v>618</v>
       </c>
       <c r="B305" t="s">
         <v>2232</v>
@@ -39675,7 +39679,7 @@
     </row>
     <row r="306" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A306">
-        <v>652</v>
+        <v>619</v>
       </c>
       <c r="B306" t="s">
         <v>2240</v>
@@ -39774,7 +39778,7 @@
     </row>
     <row r="307" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A307">
-        <v>653</v>
+        <v>620</v>
       </c>
       <c r="B307" t="s">
         <v>2249</v>
@@ -39873,7 +39877,7 @@
     </row>
     <row r="308" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A308">
-        <v>654</v>
+        <v>621</v>
       </c>
       <c r="B308" t="s">
         <v>2257</v>
@@ -39972,7 +39976,7 @@
     </row>
     <row r="309" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A309">
-        <v>655</v>
+        <v>622</v>
       </c>
       <c r="B309" t="s">
         <v>2265</v>
@@ -40071,7 +40075,7 @@
     </row>
     <row r="310" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A310">
-        <v>656</v>
+        <v>623</v>
       </c>
       <c r="B310" t="s">
         <v>2274</v>
@@ -40170,7 +40174,7 @@
     </row>
     <row r="311" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A311">
-        <v>657</v>
+        <v>624</v>
       </c>
       <c r="B311" t="s">
         <v>2286</v>
@@ -40269,7 +40273,7 @@
     </row>
     <row r="312" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A312">
-        <v>658</v>
+        <v>625</v>
       </c>
       <c r="B312" t="s">
         <v>2291</v>
@@ -40368,7 +40372,7 @@
     </row>
     <row r="313" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A313">
-        <v>659</v>
+        <v>626</v>
       </c>
       <c r="B313" t="s">
         <v>2299</v>
@@ -40467,7 +40471,7 @@
     </row>
     <row r="314" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A314">
-        <v>660</v>
+        <v>627</v>
       </c>
       <c r="B314" t="s">
         <v>2309</v>
@@ -40566,7 +40570,7 @@
     </row>
     <row r="315" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A315">
-        <v>662</v>
+        <v>628</v>
       </c>
       <c r="B315" t="s">
         <v>2319</v>
@@ -40665,7 +40669,7 @@
     </row>
     <row r="316" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A316">
-        <v>663</v>
+        <v>629</v>
       </c>
       <c r="B316" t="s">
         <v>2326</v>
@@ -40764,7 +40768,7 @@
     </row>
     <row r="317" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A317">
-        <v>664</v>
+        <v>630</v>
       </c>
       <c r="B317" t="s">
         <v>2334</v>
@@ -40863,7 +40867,7 @@
     </row>
     <row r="318" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A318">
-        <v>665</v>
+        <v>631</v>
       </c>
       <c r="B318" t="s">
         <v>2344</v>
@@ -40962,7 +40966,7 @@
     </row>
     <row r="319" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A319">
-        <v>666</v>
+        <v>632</v>
       </c>
       <c r="B319" t="s">
         <v>2351</v>
@@ -41061,7 +41065,7 @@
     </row>
     <row r="320" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A320">
-        <v>668</v>
+        <v>633</v>
       </c>
       <c r="B320" t="s">
         <v>2357</v>
@@ -41160,7 +41164,7 @@
     </row>
     <row r="321" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A321">
-        <v>669</v>
+        <v>634</v>
       </c>
       <c r="B321" t="s">
         <v>2365</v>
@@ -41259,7 +41263,7 @@
     </row>
     <row r="322" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A322">
-        <v>672</v>
+        <v>635</v>
       </c>
       <c r="B322" t="s">
         <v>2370</v>
@@ -41358,7 +41362,7 @@
     </row>
     <row r="323" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A323">
-        <v>676</v>
+        <v>637</v>
       </c>
       <c r="B323" t="s">
         <v>2376</v>
@@ -41457,7 +41461,7 @@
     </row>
     <row r="324" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A324">
-        <v>677</v>
+        <v>638</v>
       </c>
       <c r="B324" t="s">
         <v>2383</v>
@@ -41556,7 +41560,7 @@
     </row>
     <row r="325" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A325">
-        <v>679</v>
+        <v>639</v>
       </c>
       <c r="B325" t="s">
         <v>2388</v>
@@ -41655,7 +41659,7 @@
     </row>
     <row r="326" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A326">
-        <v>680</v>
+        <v>640</v>
       </c>
       <c r="B326" t="s">
         <v>2396</v>
@@ -41754,7 +41758,7 @@
     </row>
     <row r="327" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A327">
-        <v>681</v>
+        <v>641</v>
       </c>
       <c r="B327" t="s">
         <v>2402</v>
@@ -41853,7 +41857,7 @@
     </row>
     <row r="328" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A328">
-        <v>682</v>
+        <v>642</v>
       </c>
       <c r="B328" t="s">
         <v>2411</v>
@@ -41952,7 +41956,7 @@
     </row>
     <row r="329" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A329">
-        <v>684</v>
+        <v>643</v>
       </c>
       <c r="B329" t="s">
         <v>2419</v>
@@ -42051,7 +42055,7 @@
     </row>
     <row r="330" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A330">
-        <v>685</v>
+        <v>644</v>
       </c>
       <c r="B330" t="s">
         <v>2423</v>
@@ -42150,7 +42154,7 @@
     </row>
     <row r="331" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A331">
-        <v>686</v>
+        <v>645</v>
       </c>
       <c r="B331" t="s">
         <v>2431</v>
@@ -42249,7 +42253,7 @@
     </row>
     <row r="332" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A332">
-        <v>687</v>
+        <v>646</v>
       </c>
       <c r="B332" t="s">
         <v>2438</v>
@@ -42348,7 +42352,7 @@
     </row>
     <row r="333" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A333">
-        <v>688</v>
+        <v>647</v>
       </c>
       <c r="B333" t="s">
         <v>2445</v>
@@ -42447,7 +42451,7 @@
     </row>
     <row r="334" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A334">
-        <v>689</v>
+        <v>648</v>
       </c>
       <c r="B334" t="s">
         <v>2450</v>
@@ -42546,7 +42550,7 @@
     </row>
     <row r="335" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A335">
-        <v>690</v>
+        <v>649</v>
       </c>
       <c r="B335" t="s">
         <v>2457</v>
@@ -42645,7 +42649,7 @@
     </row>
     <row r="336" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A336">
-        <v>691</v>
+        <v>650</v>
       </c>
       <c r="B336" t="s">
         <v>2461</v>
@@ -42744,7 +42748,7 @@
     </row>
     <row r="337" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A337">
-        <v>692</v>
+        <v>651</v>
       </c>
       <c r="B337" t="s">
         <v>2465</v>
@@ -42843,7 +42847,7 @@
     </row>
     <row r="338" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A338">
-        <v>693</v>
+        <v>652</v>
       </c>
       <c r="B338" t="s">
         <v>2468</v>
@@ -42942,7 +42946,7 @@
     </row>
     <row r="339" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A339">
-        <v>694</v>
+        <v>653</v>
       </c>
       <c r="B339" t="s">
         <v>2472</v>
@@ -43041,7 +43045,7 @@
     </row>
     <row r="340" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A340">
-        <v>695</v>
+        <v>654</v>
       </c>
       <c r="B340" t="s">
         <v>2480</v>
@@ -43140,7 +43144,7 @@
     </row>
     <row r="341" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A341">
-        <v>696</v>
+        <v>655</v>
       </c>
       <c r="B341" t="s">
         <v>2484</v>
@@ -43239,7 +43243,7 @@
     </row>
     <row r="342" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A342">
-        <v>697</v>
+        <v>656</v>
       </c>
       <c r="B342" t="s">
         <v>2492</v>
@@ -43338,7 +43342,7 @@
     </row>
     <row r="343" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A343">
-        <v>698</v>
+        <v>657</v>
       </c>
       <c r="B343" t="s">
         <v>2500</v>
@@ -43437,7 +43441,7 @@
     </row>
     <row r="344" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A344">
-        <v>699</v>
+        <v>658</v>
       </c>
       <c r="B344" t="s">
         <v>2505</v>
@@ -43536,7 +43540,7 @@
     </row>
     <row r="345" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A345">
-        <v>700</v>
+        <v>659</v>
       </c>
       <c r="B345" t="s">
         <v>2513</v>
@@ -43635,7 +43639,7 @@
     </row>
     <row r="346" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A346">
-        <v>701</v>
+        <v>660</v>
       </c>
       <c r="B346" t="s">
         <v>2520</v>
@@ -43734,7 +43738,7 @@
     </row>
     <row r="347" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A347">
-        <v>702</v>
+        <v>661</v>
       </c>
       <c r="B347" t="s">
         <v>2530</v>
@@ -43833,7 +43837,7 @@
     </row>
     <row r="348" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A348">
-        <v>703</v>
+        <v>662</v>
       </c>
       <c r="B348" t="s">
         <v>2538</v>
@@ -43932,7 +43936,7 @@
     </row>
     <row r="349" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A349">
-        <v>704</v>
+        <v>663</v>
       </c>
       <c r="B349" t="s">
         <v>2547</v>
@@ -44031,7 +44035,7 @@
     </row>
     <row r="350" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A350">
-        <v>705</v>
+        <v>664</v>
       </c>
       <c r="B350" t="s">
         <v>2551</v>
@@ -44130,7 +44134,7 @@
     </row>
     <row r="351" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A351">
-        <v>707</v>
+        <v>665</v>
       </c>
       <c r="B351" t="s">
         <v>2557</v>
@@ -44229,7 +44233,7 @@
     </row>
     <row r="352" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A352">
-        <v>708</v>
+        <v>666</v>
       </c>
       <c r="B352" t="s">
         <v>2566</v>
@@ -44328,7 +44332,7 @@
     </row>
     <row r="353" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A353">
-        <v>709</v>
+        <v>667</v>
       </c>
       <c r="B353" t="s">
         <v>2571</v>
@@ -44427,7 +44431,7 @@
     </row>
     <row r="354" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A354">
-        <v>711</v>
+        <v>668</v>
       </c>
       <c r="B354" t="s">
         <v>2578</v>
@@ -44526,7 +44530,7 @@
     </row>
     <row r="355" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A355">
-        <v>712</v>
+        <v>669</v>
       </c>
       <c r="B355" t="s">
         <v>2583</v>
@@ -44625,7 +44629,7 @@
     </row>
     <row r="356" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A356">
-        <v>713</v>
+        <v>670</v>
       </c>
       <c r="B356" t="s">
         <v>2588</v>
@@ -44724,7 +44728,7 @@
     </row>
     <row r="357" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A357">
-        <v>715</v>
+        <v>671</v>
       </c>
       <c r="B357" t="s">
         <v>2595</v>
@@ -44822,7 +44826,7 @@
     </row>
     <row r="358" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A358">
-        <v>716</v>
+        <v>672</v>
       </c>
       <c r="B358" t="s">
         <v>2605</v>
@@ -44920,7 +44924,7 @@
     </row>
     <row r="359" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A359">
-        <v>717</v>
+        <v>673</v>
       </c>
       <c r="B359" t="s">
         <v>2610</v>
@@ -45018,7 +45022,7 @@
     </row>
     <row r="360" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A360">
-        <v>718</v>
+        <v>674</v>
       </c>
       <c r="B360" t="s">
         <v>2614</v>
@@ -45116,7 +45120,7 @@
     </row>
     <row r="361" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A361">
-        <v>719</v>
+        <v>675</v>
       </c>
       <c r="B361" t="s">
         <v>2621</v>
@@ -45214,7 +45218,7 @@
     </row>
     <row r="362" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A362">
-        <v>720</v>
+        <v>676</v>
       </c>
       <c r="B362" t="s">
         <v>2626</v>
@@ -45312,7 +45316,7 @@
     </row>
     <row r="363" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A363">
-        <v>721</v>
+        <v>677</v>
       </c>
       <c r="B363" t="s">
         <v>2634</v>
@@ -45410,7 +45414,7 @@
     </row>
     <row r="364" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A364">
-        <v>722</v>
+        <v>678</v>
       </c>
       <c r="B364" t="s">
         <v>2644</v>
@@ -45508,7 +45512,7 @@
     </row>
     <row r="365" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A365">
-        <v>723</v>
+        <v>679</v>
       </c>
       <c r="B365" t="s">
         <v>2654</v>
@@ -45606,7 +45610,7 @@
     </row>
     <row r="366" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A366">
-        <v>724</v>
+        <v>680</v>
       </c>
       <c r="B366" t="s">
         <v>2661</v>
@@ -45704,7 +45708,7 @@
     </row>
     <row r="367" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A367">
-        <v>726</v>
+        <v>681</v>
       </c>
       <c r="B367" t="s">
         <v>2672</v>
@@ -45802,7 +45806,7 @@
     </row>
     <row r="368" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A368">
-        <v>730</v>
+        <v>682</v>
       </c>
       <c r="B368" t="s">
         <v>2676</v>
@@ -45900,7 +45904,7 @@
     </row>
     <row r="369" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A369">
-        <v>731</v>
+        <v>683</v>
       </c>
       <c r="B369" t="s">
         <v>2684</v>
@@ -45998,7 +46002,7 @@
     </row>
     <row r="370" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A370">
-        <v>732</v>
+        <v>684</v>
       </c>
       <c r="B370" t="s">
         <v>2692</v>
@@ -46096,7 +46100,7 @@
     </row>
     <row r="371" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A371">
-        <v>733</v>
+        <v>685</v>
       </c>
       <c r="B371" t="s">
         <v>2695</v>
@@ -46194,7 +46198,7 @@
     </row>
     <row r="372" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A372">
-        <v>734</v>
+        <v>686</v>
       </c>
       <c r="B372" t="s">
         <v>2697</v>
@@ -46292,7 +46296,7 @@
     </row>
     <row r="373" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A373">
-        <v>735</v>
+        <v>687</v>
       </c>
       <c r="B373" t="s">
         <v>2699</v>
@@ -46390,7 +46394,7 @@
     </row>
     <row r="374" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A374">
-        <v>737</v>
+        <v>688</v>
       </c>
       <c r="B374" t="s">
         <v>2708</v>
@@ -46488,7 +46492,7 @@
     </row>
     <row r="375" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A375">
-        <v>738</v>
+        <v>689</v>
       </c>
       <c r="B375" t="s">
         <v>2718</v>
@@ -46586,7 +46590,7 @@
     </row>
     <row r="376" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A376">
-        <v>739</v>
+        <v>690</v>
       </c>
       <c r="B376" t="s">
         <v>2724</v>
@@ -46684,7 +46688,7 @@
     </row>
     <row r="377" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A377">
-        <v>741</v>
+        <v>691</v>
       </c>
       <c r="B377" t="s">
         <v>2733</v>
@@ -46782,7 +46786,7 @@
     </row>
     <row r="378" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A378">
-        <v>742</v>
+        <v>692</v>
       </c>
       <c r="B378" t="s">
         <v>2738</v>
@@ -46880,7 +46884,7 @@
     </row>
     <row r="379" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A379">
-        <v>743</v>
+        <v>693</v>
       </c>
       <c r="B379" t="s">
         <v>2745</v>
@@ -46978,7 +46982,7 @@
     </row>
     <row r="380" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A380">
-        <v>744</v>
+        <v>694</v>
       </c>
       <c r="B380" t="s">
         <v>2750</v>
@@ -47076,7 +47080,7 @@
     </row>
     <row r="381" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A381">
-        <v>745</v>
+        <v>695</v>
       </c>
       <c r="B381" t="s">
         <v>2755</v>
@@ -47174,7 +47178,7 @@
     </row>
     <row r="382" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A382">
-        <v>746</v>
+        <v>696</v>
       </c>
       <c r="B382" t="s">
         <v>2760</v>
@@ -47272,7 +47276,7 @@
     </row>
     <row r="383" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A383">
-        <v>748</v>
+        <v>697</v>
       </c>
       <c r="B383" t="s">
         <v>2770</v>
@@ -47370,7 +47374,7 @@
     </row>
     <row r="384" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A384">
-        <v>749</v>
+        <v>698</v>
       </c>
       <c r="B384" t="s">
         <v>2775</v>
@@ -47468,7 +47472,7 @@
     </row>
     <row r="385" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A385">
-        <v>751</v>
+        <v>699</v>
       </c>
       <c r="B385" t="s">
         <v>2782</v>
@@ -47566,7 +47570,7 @@
     </row>
     <row r="386" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A386">
-        <v>752</v>
+        <v>700</v>
       </c>
       <c r="B386" t="s">
         <v>2789</v>
@@ -47664,7 +47668,7 @@
     </row>
     <row r="387" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A387">
-        <v>753</v>
+        <v>701</v>
       </c>
       <c r="B387" t="s">
         <v>2798</v>
@@ -47762,7 +47766,7 @@
     </row>
     <row r="388" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A388">
-        <v>755</v>
+        <v>702</v>
       </c>
       <c r="B388" t="s">
         <v>2808</v>
@@ -47860,7 +47864,7 @@
     </row>
     <row r="389" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A389">
-        <v>756</v>
+        <v>703</v>
       </c>
       <c r="B389" t="s">
         <v>2819</v>
@@ -47958,7 +47962,7 @@
     </row>
     <row r="390" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A390">
-        <v>757</v>
+        <v>704</v>
       </c>
       <c r="B390" t="s">
         <v>2829</v>
@@ -48056,7 +48060,7 @@
     </row>
     <row r="391" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A391">
-        <v>758</v>
+        <v>705</v>
       </c>
       <c r="B391" t="s">
         <v>2836</v>
@@ -48154,7 +48158,7 @@
     </row>
     <row r="392" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A392">
-        <v>760</v>
+        <v>706</v>
       </c>
       <c r="B392" t="s">
         <v>2846</v>
@@ -48252,7 +48256,7 @@
     </row>
     <row r="393" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A393">
-        <v>761</v>
+        <v>707</v>
       </c>
       <c r="B393" t="s">
         <v>2856</v>
@@ -48350,7 +48354,7 @@
     </row>
     <row r="394" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A394">
-        <v>762</v>
+        <v>708</v>
       </c>
       <c r="B394" t="s">
         <v>2865</v>
@@ -48448,7 +48452,7 @@
     </row>
     <row r="395" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A395">
-        <v>763</v>
+        <v>709</v>
       </c>
       <c r="B395" t="s">
         <v>2874</v>
@@ -48546,7 +48550,7 @@
     </row>
     <row r="396" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A396">
-        <v>764</v>
+        <v>710</v>
       </c>
       <c r="B396" t="s">
         <v>2880</v>
@@ -48644,7 +48648,7 @@
     </row>
     <row r="397" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A397">
-        <v>765</v>
+        <v>711</v>
       </c>
       <c r="B397" t="s">
         <v>2891</v>
@@ -48742,7 +48746,7 @@
     </row>
     <row r="398" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A398">
-        <v>766</v>
+        <v>712</v>
       </c>
       <c r="B398" t="s">
         <v>2897</v>
@@ -48840,7 +48844,7 @@
     </row>
     <row r="399" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A399">
-        <v>767</v>
+        <v>713</v>
       </c>
       <c r="B399" t="s">
         <v>2899</v>
@@ -48938,7 +48942,7 @@
     </row>
     <row r="400" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A400">
-        <v>768</v>
+        <v>714</v>
       </c>
       <c r="B400" t="s">
         <v>2909</v>
@@ -49036,7 +49040,7 @@
     </row>
     <row r="401" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A401">
-        <v>769</v>
+        <v>715</v>
       </c>
       <c r="B401" t="s">
         <v>2919</v>
@@ -49134,7 +49138,7 @@
     </row>
     <row r="402" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A402">
-        <v>770</v>
+        <v>716</v>
       </c>
       <c r="B402" t="s">
         <v>2924</v>
@@ -49232,7 +49236,7 @@
     </row>
     <row r="403" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A403">
-        <v>771</v>
+        <v>717</v>
       </c>
       <c r="B403" t="s">
         <v>2927</v>
@@ -49330,7 +49334,7 @@
     </row>
     <row r="404" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A404">
-        <v>772</v>
+        <v>718</v>
       </c>
       <c r="B404" t="s">
         <v>2933</v>
@@ -49428,7 +49432,7 @@
     </row>
     <row r="405" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A405">
-        <v>774</v>
+        <v>719</v>
       </c>
       <c r="B405" t="s">
         <v>2938</v>
@@ -49526,7 +49530,7 @@
     </row>
     <row r="406" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A406">
-        <v>775</v>
+        <v>720</v>
       </c>
       <c r="B406" t="s">
         <v>2943</v>
@@ -49624,7 +49628,7 @@
     </row>
     <row r="407" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A407">
-        <v>776</v>
+        <v>721</v>
       </c>
       <c r="B407" t="s">
         <v>2949</v>
@@ -49722,7 +49726,7 @@
     </row>
     <row r="408" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A408">
-        <v>777</v>
+        <v>722</v>
       </c>
       <c r="B408" t="s">
         <v>2959</v>
@@ -49820,7 +49824,7 @@
     </row>
     <row r="409" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A409">
-        <v>778</v>
+        <v>723</v>
       </c>
       <c r="B409" t="s">
         <v>2967</v>
@@ -49918,7 +49922,7 @@
     </row>
     <row r="410" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A410">
-        <v>750</v>
+        <v>724</v>
       </c>
       <c r="B410" t="s">
         <v>2971</v>

</xml_diff>

<commit_message>
Commit: Fecha_inicio_contrato like fecha_inicio.
</commit_message>
<xml_diff>
--- a/data/input/base_contratos.xlsx
+++ b/data/input/base_contratos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Soriana\00 - AUDITORIA 2020 - 2024\00 - Auditores\Oscar\Proyectos Python\Automation-Subarrenda\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473E6EB5-2D16-47F6-B8AA-D00507BA2A34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17C4BE1D-BF9A-482C-A075-13FDCDD532C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15840" xr2:uid="{0E8B9EC1-6715-4F8D-BBDE-46BF36F37EC3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9505" uniqueCount="2975">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9504" uniqueCount="2974">
   <si>
     <t>orden</t>
   </si>
@@ -8964,9 +8964,6 @@
   </si>
   <si>
     <t>208.50 METROS CUADRADOS</t>
-  </si>
-  <si>
-    <t>15/1/2015</t>
   </si>
 </sst>
 </file>
@@ -33948,8 +33945,8 @@
       <c r="D248" t="s">
         <v>1814</v>
       </c>
-      <c r="F248" s="1" t="s">
-        <v>2974</v>
+      <c r="F248" s="1">
+        <v>42019</v>
       </c>
       <c r="G248" s="1">
         <v>47285</v>

</xml_diff>

<commit_message>
feat: Update base_cliente and base_contratos Excel files
</commit_message>
<xml_diff>
--- a/data/input/base_contratos.xlsx
+++ b/data/input/base_contratos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Soriana\00 - AUDITORIA 2020 - 2024\00 - Auditores\Oscar\Proyectos Python\Automation-Subarrenda\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17C4BE1D-BF9A-482C-A075-13FDCDD532C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B4DD21-2E4D-4A87-A87F-F0AF5F3611A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15840" xr2:uid="{0E8B9EC1-6715-4F8D-BBDE-46BF36F37EC3}"/>
   </bookViews>
@@ -9344,6 +9344,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="24.42578125" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>
@@ -9781,10 +9782,10 @@
         <v>55</v>
       </c>
       <c r="F5" s="1">
-        <v>45628</v>
+        <v>45627</v>
       </c>
       <c r="G5" s="1">
-        <v>45505</v>
+        <v>50009</v>
       </c>
       <c r="H5" t="s">
         <v>76</v>
@@ -10702,7 +10703,7 @@
         <v>45505</v>
       </c>
       <c r="G14" s="1">
-        <v>45504</v>
+        <v>46599</v>
       </c>
       <c r="H14" t="s">
         <v>148</v>
@@ -10801,10 +10802,10 @@
         <v>64</v>
       </c>
       <c r="F15" s="1">
+        <v>44469</v>
+      </c>
+      <c r="G15" s="1">
         <v>46659</v>
-      </c>
-      <c r="G15" s="1">
-        <v>48497</v>
       </c>
       <c r="H15" t="s">
         <v>42</v>
@@ -12436,7 +12437,7 @@
         <v>44625</v>
       </c>
       <c r="G31" s="1">
-        <v>43710</v>
+        <v>45720</v>
       </c>
       <c r="H31" t="s">
         <v>294</v>
@@ -13252,7 +13253,7 @@
         <v>45413</v>
       </c>
       <c r="G39" s="1">
-        <v>43668</v>
+        <v>45777</v>
       </c>
       <c r="H39">
         <v>1916889124</v>
@@ -13354,7 +13355,7 @@
         <v>45230</v>
       </c>
       <c r="G40" s="1">
-        <v>45202</v>
+        <v>47026</v>
       </c>
       <c r="H40" t="s">
         <v>359</v>
@@ -22069,7 +22070,7 @@
         <v>45505</v>
       </c>
       <c r="G128" s="1">
-        <v>44960</v>
+        <v>46053</v>
       </c>
       <c r="H128" t="s">
         <v>513</v>
@@ -23242,7 +23243,7 @@
     </row>
     <row r="140" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A140">
-        <v>464</v>
+        <v>725</v>
       </c>
       <c r="B140" t="s">
         <v>953</v>
@@ -38107,7 +38108,7 @@
         <v>44896</v>
       </c>
       <c r="G290" s="1">
-        <v>40725</v>
+        <v>47968</v>
       </c>
       <c r="H290" t="s">
         <v>2129</v>

</xml_diff>